<commit_message>
Update Shopee listing data: 8.5 mass update files and price sheet
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shopee上架/TrinityGlobe_Shopee_upload.xlsx
+++ b/shopee上架/TrinityGlobe_Shopee_upload.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hengchangqi/Documents/Singapore/Plan &amp; Note Internship/Part Time/WeChatProjects/TrinityGlobe/shopee上架/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77F6657B-B78A-6A49-8D69-499DCD0933E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1FE4668-D5E9-1C4B-9145-14C4CAF74079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1460" yWindow="660" windowWidth="25680" windowHeight="16560" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,20 @@
     <sheet name="HiddenShopBrand" sheetId="6" state="hidden" r:id="rId6"/>
     <sheet name="HiddenTax" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -12186,13 +12199,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
@@ -12203,16 +12209,23 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
@@ -12504,591 +12517,563 @@
     <row r="1" spans="1:14" ht="15" hidden="1" customHeight="1"/>
     <row r="2" spans="1:14" ht="15" hidden="1" customHeight="1"/>
     <row r="3" spans="1:14" ht="25" customHeight="1">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="13"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
     </row>
     <row r="4" spans="1:14" ht="15" customHeight="1">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
     </row>
     <row r="5" spans="1:14" ht="15" customHeight="1">
-      <c r="A5" s="11"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
+      <c r="A5" s="12"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="12"/>
+      <c r="L5" s="12"/>
+      <c r="M5" s="12"/>
+      <c r="N5" s="12"/>
     </row>
     <row r="6" spans="1:14" ht="15" customHeight="1">
-      <c r="A6" s="11"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
+      <c r="A6" s="12"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="12"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
     </row>
     <row r="7" spans="1:14" ht="15" customHeight="1">
-      <c r="A7" s="11"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11"/>
+      <c r="A7" s="12"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="12"/>
+      <c r="M7" s="12"/>
+      <c r="N7" s="12"/>
     </row>
     <row r="8" spans="1:14" ht="15" customHeight="1">
-      <c r="A8" s="11"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="11"/>
+      <c r="A8" s="12"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="12"/>
+      <c r="M8" s="12"/>
+      <c r="N8" s="12"/>
     </row>
     <row r="9" spans="1:14" ht="15" customHeight="1">
-      <c r="A9" s="11"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
+      <c r="A9" s="12"/>
+      <c r="B9" s="12"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="12"/>
+      <c r="N9" s="12"/>
     </row>
     <row r="10" spans="1:14" ht="25" customHeight="1">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="13"/>
-      <c r="L10" s="13"/>
-      <c r="M10" s="13"/>
-      <c r="N10" s="13"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
     </row>
     <row r="11" spans="1:14" ht="15" customHeight="1">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="11"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12"/>
     </row>
     <row r="12" spans="1:14" ht="15" customHeight="1">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="11"/>
-      <c r="N12" s="11"/>
+      <c r="A12" s="12"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="12"/>
+      <c r="M12" s="12"/>
+      <c r="N12" s="12"/>
     </row>
     <row r="13" spans="1:14" ht="15" customHeight="1">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
+      <c r="A13" s="12"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="12"/>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12"/>
     </row>
     <row r="14" spans="1:14" ht="15" customHeight="1">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="11"/>
+      <c r="A14" s="12"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="12"/>
+      <c r="L14" s="12"/>
+      <c r="M14" s="12"/>
+      <c r="N14" s="12"/>
     </row>
     <row r="15" spans="1:14" ht="25" customHeight="1">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
-      <c r="J15" s="13"/>
-      <c r="K15" s="13"/>
-      <c r="L15" s="13"/>
-      <c r="M15" s="13"/>
-      <c r="N15" s="13"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
     </row>
     <row r="16" spans="1:14" ht="15" customHeight="1">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="11"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="12"/>
+      <c r="L16" s="12"/>
+      <c r="M16" s="12"/>
+      <c r="N16" s="12"/>
     </row>
     <row r="17" spans="1:14" ht="15" customHeight="1">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="11"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
     </row>
     <row r="18" spans="1:14" ht="15" customHeight="1">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="12"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12"/>
     </row>
     <row r="19" spans="1:14" ht="15" customHeight="1">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="11"/>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11"/>
-      <c r="N19" s="11"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="12"/>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12"/>
     </row>
     <row r="20" spans="1:14" ht="15" customHeight="1">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="11"/>
-      <c r="L20" s="11"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="11"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
+      <c r="L20" s="12"/>
+      <c r="M20" s="12"/>
+      <c r="N20" s="12"/>
     </row>
     <row r="21" spans="1:14" ht="15" customHeight="1">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="12"/>
+      <c r="M21" s="12"/>
+      <c r="N21" s="12"/>
     </row>
     <row r="22" spans="1:14" ht="15" customHeight="1">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11"/>
-      <c r="L22" s="11"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="12"/>
+      <c r="L22" s="12"/>
+      <c r="M22" s="12"/>
+      <c r="N22" s="12"/>
     </row>
     <row r="23" spans="1:14" ht="15" customHeight="1">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="11"/>
-      <c r="L23" s="11"/>
-      <c r="M23" s="11"/>
-      <c r="N23" s="11"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="12"/>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12"/>
     </row>
     <row r="24" spans="1:14" ht="15" customHeight="1">
-      <c r="A24" s="9" t="s">
+      <c r="A24" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11"/>
-      <c r="L24" s="11"/>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="12"/>
+      <c r="L24" s="12"/>
+      <c r="M24" s="12"/>
+      <c r="N24" s="12"/>
     </row>
     <row r="25" spans="1:14" ht="15" customHeight="1">
-      <c r="A25" s="9" t="s">
+      <c r="A25" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="12"/>
+      <c r="M25" s="12"/>
+      <c r="N25" s="12"/>
     </row>
     <row r="26" spans="1:14" ht="15" customHeight="1">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="11"/>
-      <c r="J26" s="11"/>
-      <c r="K26" s="11"/>
-      <c r="L26" s="11"/>
-      <c r="M26" s="11"/>
-      <c r="N26" s="11"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="12"/>
+      <c r="L26" s="12"/>
+      <c r="M26" s="12"/>
+      <c r="N26" s="12"/>
     </row>
     <row r="27" spans="1:14" ht="25" customHeight="1">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="13"/>
-      <c r="H27" s="13"/>
-      <c r="I27" s="13"/>
-      <c r="J27" s="13"/>
-      <c r="K27" s="13"/>
-      <c r="L27" s="13"/>
-      <c r="M27" s="13"/>
-      <c r="N27" s="13"/>
+      <c r="B27" s="10"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="10"/>
+      <c r="L27" s="10"/>
+      <c r="M27" s="10"/>
+      <c r="N27" s="10"/>
     </row>
     <row r="28" spans="1:14" ht="15" customHeight="1">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="11"/>
-      <c r="J28" s="11"/>
-      <c r="K28" s="11"/>
-      <c r="L28" s="11"/>
-      <c r="M28" s="11"/>
-      <c r="N28" s="11"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+      <c r="I28" s="12"/>
+      <c r="J28" s="12"/>
+      <c r="K28" s="12"/>
+      <c r="L28" s="12"/>
+      <c r="M28" s="12"/>
+      <c r="N28" s="12"/>
     </row>
     <row r="29" spans="1:14" ht="15" customHeight="1">
-      <c r="A29" s="9" t="s">
+      <c r="A29" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="11"/>
-      <c r="J29" s="11"/>
-      <c r="K29" s="11"/>
-      <c r="L29" s="11"/>
-      <c r="M29" s="11"/>
-      <c r="N29" s="11"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="12"/>
+      <c r="L29" s="12"/>
+      <c r="M29" s="12"/>
+      <c r="N29" s="12"/>
     </row>
     <row r="30" spans="1:14" ht="15" customHeight="1">
-      <c r="A30" s="9" t="s">
+      <c r="A30" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-      <c r="G30" s="11"/>
-      <c r="H30" s="11"/>
-      <c r="I30" s="11"/>
-      <c r="J30" s="11"/>
-      <c r="K30" s="11"/>
-      <c r="L30" s="11"/>
-      <c r="M30" s="11"/>
-      <c r="N30" s="11"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="12"/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="12"/>
+      <c r="L30" s="12"/>
+      <c r="M30" s="12"/>
+      <c r="N30" s="12"/>
     </row>
     <row r="31" spans="1:14" ht="15" customHeight="1">
-      <c r="A31" s="9" t="s">
+      <c r="A31" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="11"/>
-      <c r="J31" s="11"/>
-      <c r="K31" s="11"/>
-      <c r="L31" s="11"/>
-      <c r="M31" s="11"/>
-      <c r="N31" s="11"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="12"/>
+      <c r="K31" s="12"/>
+      <c r="L31" s="12"/>
+      <c r="M31" s="12"/>
+      <c r="N31" s="12"/>
     </row>
     <row r="32" spans="1:14" ht="15" customHeight="1">
-      <c r="A32" s="9" t="s">
+      <c r="A32" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="B32" s="10" t="s">
+      <c r="B32" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="11"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="11"/>
-      <c r="J32" s="11"/>
-      <c r="K32" s="11"/>
-      <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
-      <c r="N32" s="11"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="12"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="12"/>
+      <c r="J32" s="12"/>
+      <c r="K32" s="12"/>
+      <c r="L32" s="12"/>
+      <c r="M32" s="12"/>
+      <c r="N32" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="A3:N3"/>
-    <mergeCell ref="A4:N9"/>
-    <mergeCell ref="A10:N10"/>
-    <mergeCell ref="A11:N14"/>
-    <mergeCell ref="A15:N15"/>
-    <mergeCell ref="A16"/>
-    <mergeCell ref="B16:N16"/>
-    <mergeCell ref="A17"/>
-    <mergeCell ref="B17:N17"/>
-    <mergeCell ref="A18"/>
-    <mergeCell ref="B18:N18"/>
-    <mergeCell ref="A19"/>
-    <mergeCell ref="B19:N19"/>
-    <mergeCell ref="A20"/>
-    <mergeCell ref="B20:N20"/>
-    <mergeCell ref="A21"/>
-    <mergeCell ref="B21:N21"/>
-    <mergeCell ref="A22"/>
-    <mergeCell ref="B22:N22"/>
-    <mergeCell ref="A23"/>
-    <mergeCell ref="B23:N23"/>
-    <mergeCell ref="A24"/>
-    <mergeCell ref="B24:N24"/>
-    <mergeCell ref="A25"/>
-    <mergeCell ref="B25:N25"/>
-    <mergeCell ref="A26"/>
-    <mergeCell ref="B26:N26"/>
-    <mergeCell ref="A27:N27"/>
     <mergeCell ref="A31"/>
     <mergeCell ref="B31:N31"/>
     <mergeCell ref="A32"/>
@@ -13099,6 +13084,34 @@
     <mergeCell ref="B29:N29"/>
     <mergeCell ref="A30"/>
     <mergeCell ref="B30:N30"/>
+    <mergeCell ref="A25"/>
+    <mergeCell ref="B25:N25"/>
+    <mergeCell ref="A26"/>
+    <mergeCell ref="B26:N26"/>
+    <mergeCell ref="A27:N27"/>
+    <mergeCell ref="A22"/>
+    <mergeCell ref="B22:N22"/>
+    <mergeCell ref="A23"/>
+    <mergeCell ref="B23:N23"/>
+    <mergeCell ref="A24"/>
+    <mergeCell ref="B24:N24"/>
+    <mergeCell ref="A19"/>
+    <mergeCell ref="B19:N19"/>
+    <mergeCell ref="A20"/>
+    <mergeCell ref="B20:N20"/>
+    <mergeCell ref="A21"/>
+    <mergeCell ref="B21:N21"/>
+    <mergeCell ref="A16"/>
+    <mergeCell ref="B16:N16"/>
+    <mergeCell ref="A17"/>
+    <mergeCell ref="B17:N17"/>
+    <mergeCell ref="A18"/>
+    <mergeCell ref="B18:N18"/>
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A4:N9"/>
+    <mergeCell ref="A10:N10"/>
+    <mergeCell ref="A11:N14"/>
+    <mergeCell ref="A15:N15"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16905,132 +16918,132 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:47" hidden="1">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>321</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="12" t="s">
         <v>322</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="12" t="s">
         <v>323</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="12" t="s">
         <v>324</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="12" t="s">
         <v>325</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="12" t="s">
         <v>326</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="12" t="s">
         <v>327</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="12" t="s">
         <v>328</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="12" t="s">
         <v>329</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="12" t="s">
         <v>330</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="12" t="s">
         <v>331</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="12" t="s">
         <v>332</v>
       </c>
-      <c r="M1" s="11" t="s">
+      <c r="M1" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="N1" s="11" t="s">
+      <c r="N1" s="12" t="s">
         <v>334</v>
       </c>
-      <c r="O1" s="11" t="s">
+      <c r="O1" s="12" t="s">
         <v>335</v>
       </c>
-      <c r="P1" s="11" t="s">
+      <c r="P1" s="12" t="s">
         <v>336</v>
       </c>
-      <c r="Q1" s="11" t="s">
+      <c r="Q1" s="12" t="s">
         <v>337</v>
       </c>
-      <c r="R1" s="11" t="s">
+      <c r="R1" s="12" t="s">
         <v>338</v>
       </c>
-      <c r="S1" s="11" t="s">
+      <c r="S1" s="12" t="s">
         <v>339</v>
       </c>
-      <c r="T1" s="11" t="s">
+      <c r="T1" s="12" t="s">
         <v>340</v>
       </c>
-      <c r="U1" s="11" t="s">
+      <c r="U1" s="12" t="s">
         <v>341</v>
       </c>
-      <c r="V1" s="11" t="s">
+      <c r="V1" s="12" t="s">
         <v>342</v>
       </c>
-      <c r="W1" s="11" t="s">
+      <c r="W1" s="12" t="s">
         <v>343</v>
       </c>
-      <c r="X1" s="11" t="s">
+      <c r="X1" s="12" t="s">
         <v>344</v>
       </c>
-      <c r="Y1" s="11" t="s">
+      <c r="Y1" s="12" t="s">
         <v>345</v>
       </c>
-      <c r="Z1" s="11" t="s">
+      <c r="Z1" s="12" t="s">
         <v>346</v>
       </c>
-      <c r="AA1" s="11" t="s">
+      <c r="AA1" s="12" t="s">
         <v>347</v>
       </c>
-      <c r="AB1" s="11" t="s">
+      <c r="AB1" s="12" t="s">
         <v>348</v>
       </c>
-      <c r="AC1" s="11" t="s">
+      <c r="AC1" s="12" t="s">
         <v>349</v>
       </c>
-      <c r="AD1" s="11" t="s">
+      <c r="AD1" s="12" t="s">
         <v>349</v>
       </c>
-      <c r="AE1" s="11" t="s">
+      <c r="AE1" s="12" t="s">
         <v>349</v>
       </c>
-      <c r="AF1" s="11" t="s">
+      <c r="AF1" s="12" t="s">
         <v>350</v>
       </c>
-      <c r="AG1" s="11" t="s">
+      <c r="AG1" s="12" t="s">
         <v>351</v>
       </c>
-      <c r="AH1" s="11" t="s">
+      <c r="AH1" s="12" t="s">
         <v>352</v>
       </c>
-      <c r="AI1" s="11"/>
-      <c r="AJ1" s="11"/>
-      <c r="AK1" s="11"/>
-      <c r="AL1" s="11"/>
-      <c r="AM1" s="11"/>
-      <c r="AN1" s="11"/>
-      <c r="AO1" s="11"/>
-      <c r="AP1" s="11"/>
-      <c r="AQ1" s="11"/>
-      <c r="AR1" s="11" t="s">
+      <c r="AI1" s="12"/>
+      <c r="AJ1" s="12"/>
+      <c r="AK1" s="12"/>
+      <c r="AL1" s="12"/>
+      <c r="AM1" s="12"/>
+      <c r="AN1" s="12"/>
+      <c r="AO1" s="12"/>
+      <c r="AP1" s="12"/>
+      <c r="AQ1" s="12"/>
+      <c r="AR1" s="12" t="s">
         <v>353</v>
       </c>
-      <c r="AS1" s="11" t="s">
+      <c r="AS1" s="12" t="s">
         <v>354</v>
       </c>
-      <c r="AT1" s="11" t="s">
+      <c r="AT1" s="12" t="s">
         <v>355</v>
       </c>
-      <c r="AU1" s="11" t="s">
+      <c r="AU1" s="12" t="s">
         <v>356</v>
       </c>
     </row>
     <row r="2" spans="1:47" hidden="1">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="12" t="s">
         <v>73</v>
       </c>
     </row>
@@ -17181,49 +17194,49 @@
       <c r="A4" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="16" t="s">
         <v>109</v>
       </c>
       <c r="D4" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="J4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="K4" s="18" t="s">
+      <c r="K4" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="L4" s="18" t="s">
+      <c r="L4" s="16" t="s">
         <v>109</v>
       </c>
       <c r="M4" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="N4" s="18" t="s">
+      <c r="N4" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="O4" s="18" t="s">
+      <c r="O4" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="P4" s="18" t="s">
+      <c r="P4" s="16" t="s">
         <v>109</v>
       </c>
       <c r="Q4" s="17" t="s">
@@ -17250,7 +17263,7 @@
       <c r="X4" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="Y4" s="18" t="s">
+      <c r="Y4" s="16" t="s">
         <v>109</v>
       </c>
       <c r="Z4" s="17" t="s">
@@ -17262,13 +17275,13 @@
       <c r="AB4" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="AC4" s="16" t="s">
+      <c r="AC4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="AD4" s="16" t="s">
+      <c r="AD4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="AE4" s="16" t="s">
+      <c r="AE4" s="18" t="s">
         <v>110</v>
       </c>
       <c r="AF4" s="17" t="s">
@@ -17277,46 +17290,46 @@
       <c r="AG4" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="AH4" s="18" t="s">
+      <c r="AH4" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="AI4" s="16" t="s">
+      <c r="AI4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="AJ4" s="16" t="s">
+      <c r="AJ4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="AK4" s="16" t="s">
+      <c r="AK4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="AL4" s="16" t="s">
+      <c r="AL4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="AM4" s="16" t="s">
+      <c r="AM4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="AN4" s="16" t="s">
+      <c r="AN4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="AO4" s="16" t="s">
+      <c r="AO4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="AP4" s="16" t="s">
+      <c r="AP4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="AQ4" s="16" t="s">
+      <c r="AQ4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="AR4" s="18" t="s">
+      <c r="AR4" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="AS4" s="18" t="s">
+      <c r="AS4" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="AT4" s="16" t="s">
+      <c r="AT4" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="AU4" s="16" t="s">
+      <c r="AU4" s="18" t="s">
         <v>110</v>
       </c>
     </row>
@@ -17591,413 +17604,413 @@
       </c>
     </row>
     <row r="7" spans="1:47" ht="40" customHeight="1">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="12" t="s">
         <v>423</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="12" t="s">
         <v>424</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="12" t="s">
         <v>425</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="12" t="s">
         <v>426</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="12" t="s">
         <v>427</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="12" t="s">
         <v>428</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="H7" s="12" t="s">
         <v>429</v>
       </c>
-      <c r="I7" s="11" t="s">
+      <c r="I7" s="12" t="s">
         <v>430</v>
       </c>
-      <c r="J7" s="11" t="s">
+      <c r="J7" s="12" t="s">
         <v>431</v>
       </c>
-      <c r="K7" s="11" t="s">
+      <c r="K7" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="L7" s="11" t="s">
+      <c r="L7" s="12" t="s">
         <v>432</v>
       </c>
-      <c r="M7" s="11" t="s">
+      <c r="M7" s="12" t="s">
         <v>433</v>
       </c>
-      <c r="N7" s="11" t="s">
+      <c r="N7" s="12" t="s">
         <v>434</v>
       </c>
-      <c r="O7" s="11" t="s">
+      <c r="O7" s="12" t="s">
         <v>435</v>
       </c>
-      <c r="P7" s="11" t="s">
+      <c r="P7" s="12" t="s">
         <v>429</v>
       </c>
-      <c r="Y7" s="11" t="s">
+      <c r="Y7" s="12" t="s">
         <v>436</v>
       </c>
-      <c r="AC7" s="11" t="s">
+      <c r="AC7" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AD7" s="11" t="s">
+      <c r="AD7" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AE7" s="11" t="s">
+      <c r="AE7" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AF7" s="11" t="s">
+      <c r="AF7" s="12" t="s">
         <v>437</v>
       </c>
-      <c r="AH7" s="11" t="s">
+      <c r="AH7" s="12" t="s">
         <v>438</v>
       </c>
       <c r="AI7" s="19"/>
       <c r="AJ7" s="19"/>
-      <c r="AK7" s="11" t="s">
+      <c r="AK7" s="12" t="s">
         <v>439</v>
       </c>
       <c r="AL7" s="19"/>
       <c r="AM7" s="19"/>
-      <c r="AN7" s="11" t="s">
+      <c r="AN7" s="12" t="s">
         <v>440</v>
       </c>
       <c r="AO7" s="19"/>
       <c r="AP7" s="19"/>
       <c r="AQ7" s="19"/>
-      <c r="AR7" s="11" t="s">
+      <c r="AR7" s="12" t="s">
         <v>441</v>
       </c>
-      <c r="AS7" s="11" t="s">
+      <c r="AS7" s="12" t="s">
         <v>442</v>
       </c>
-      <c r="AT7" s="11" t="s">
+      <c r="AT7" s="12" t="s">
         <v>443</v>
       </c>
-      <c r="AU7" s="11" t="s">
+      <c r="AU7" s="12" t="s">
         <v>444</v>
       </c>
     </row>
     <row r="8" spans="1:47" ht="40" customHeight="1">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="12" t="s">
         <v>423</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="12" t="s">
         <v>424</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="12" t="s">
         <v>425</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="12" t="s">
         <v>426</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="12" t="s">
         <v>427</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="12" t="s">
         <v>428</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="12" t="s">
         <v>445</v>
       </c>
-      <c r="I8" s="11" t="s">
+      <c r="I8" s="12" t="s">
         <v>430</v>
       </c>
-      <c r="J8" s="11" t="s">
+      <c r="J8" s="12" t="s">
         <v>446</v>
       </c>
-      <c r="K8" s="11" t="s">
+      <c r="K8" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="L8" s="11" t="s">
+      <c r="L8" s="12" t="s">
         <v>432</v>
       </c>
-      <c r="M8" s="11" t="s">
+      <c r="M8" s="12" t="s">
         <v>447</v>
       </c>
-      <c r="N8" s="11" t="s">
+      <c r="N8" s="12" t="s">
         <v>448</v>
       </c>
-      <c r="O8" s="11" t="s">
+      <c r="O8" s="12" t="s">
         <v>449</v>
       </c>
-      <c r="P8" s="11" t="s">
+      <c r="P8" s="12" t="s">
         <v>445</v>
       </c>
-      <c r="Y8" s="11" t="s">
+      <c r="Y8" s="12" t="s">
         <v>436</v>
       </c>
-      <c r="AC8" s="11" t="s">
+      <c r="AC8" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AD8" s="11" t="s">
+      <c r="AD8" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AE8" s="11" t="s">
+      <c r="AE8" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AF8" s="11" t="s">
+      <c r="AF8" s="12" t="s">
         <v>437</v>
       </c>
-      <c r="AH8" s="11" t="s">
+      <c r="AH8" s="12" t="s">
         <v>438</v>
       </c>
       <c r="AI8" s="19"/>
       <c r="AJ8" s="19"/>
-      <c r="AK8" s="11" t="s">
+      <c r="AK8" s="12" t="s">
         <v>450</v>
       </c>
       <c r="AL8" s="19"/>
       <c r="AM8" s="19"/>
-      <c r="AN8" s="11" t="s">
+      <c r="AN8" s="12" t="s">
         <v>440</v>
       </c>
       <c r="AO8" s="19"/>
       <c r="AP8" s="19"/>
       <c r="AQ8" s="19"/>
-      <c r="AR8" s="11" t="s">
+      <c r="AR8" s="12" t="s">
         <v>451</v>
       </c>
-      <c r="AS8" s="11" t="s">
+      <c r="AS8" s="12" t="s">
         <v>442</v>
       </c>
-      <c r="AT8" s="11" t="s">
+      <c r="AT8" s="12" t="s">
         <v>443</v>
       </c>
-      <c r="AU8" s="11" t="s">
+      <c r="AU8" s="12" t="s">
         <v>444</v>
       </c>
     </row>
     <row r="9" spans="1:47" ht="40" customHeight="1">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="12" t="s">
         <v>423</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="12" t="s">
         <v>424</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="12" t="s">
         <v>425</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="12" t="s">
         <v>426</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="12" t="s">
         <v>427</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="12" t="s">
         <v>452</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="H9" s="12" t="s">
         <v>429</v>
       </c>
-      <c r="I9" s="11" t="s">
+      <c r="I9" s="12" t="s">
         <v>430</v>
       </c>
-      <c r="J9" s="11" t="s">
+      <c r="J9" s="12" t="s">
         <v>453</v>
       </c>
-      <c r="K9" s="11" t="s">
+      <c r="K9" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="L9" s="11" t="s">
+      <c r="L9" s="12" t="s">
         <v>432</v>
       </c>
-      <c r="M9" s="11" t="s">
+      <c r="M9" s="12" t="s">
         <v>454</v>
       </c>
-      <c r="N9" s="11" t="s">
+      <c r="N9" s="12" t="s">
         <v>455</v>
       </c>
-      <c r="O9" s="11" t="s">
+      <c r="O9" s="12" t="s">
         <v>456</v>
       </c>
-      <c r="P9" s="11" t="s">
+      <c r="P9" s="12" t="s">
         <v>445</v>
       </c>
-      <c r="Y9" s="11" t="s">
+      <c r="Y9" s="12" t="s">
         <v>436</v>
       </c>
-      <c r="AC9" s="11" t="s">
+      <c r="AC9" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AD9" s="11" t="s">
+      <c r="AD9" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AE9" s="11" t="s">
+      <c r="AE9" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AF9" s="11" t="s">
+      <c r="AF9" s="12" t="s">
         <v>437</v>
       </c>
-      <c r="AH9" s="11" t="s">
+      <c r="AH9" s="12" t="s">
         <v>438</v>
       </c>
       <c r="AI9" s="19"/>
       <c r="AJ9" s="19"/>
-      <c r="AK9" s="11" t="s">
+      <c r="AK9" s="12" t="s">
         <v>457</v>
       </c>
       <c r="AL9" s="19"/>
       <c r="AM9" s="19"/>
-      <c r="AN9" s="11" t="s">
+      <c r="AN9" s="12" t="s">
         <v>440</v>
       </c>
       <c r="AO9" s="19"/>
       <c r="AP9" s="19"/>
       <c r="AQ9" s="19"/>
-      <c r="AR9" s="11" t="s">
+      <c r="AR9" s="12" t="s">
         <v>458</v>
       </c>
-      <c r="AS9" s="11" t="s">
+      <c r="AS9" s="12" t="s">
         <v>442</v>
       </c>
-      <c r="AT9" s="11" t="s">
+      <c r="AT9" s="12" t="s">
         <v>443</v>
       </c>
-      <c r="AU9" s="11" t="s">
+      <c r="AU9" s="12" t="s">
         <v>444</v>
       </c>
     </row>
     <row r="10" spans="1:47" ht="40" customHeight="1">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="12" t="s">
         <v>459</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="12" t="s">
         <v>460</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="12" t="s">
         <v>461</v>
       </c>
-      <c r="K10" s="11" t="s">
+      <c r="K10" s="12" t="s">
         <v>462</v>
       </c>
-      <c r="L10" s="11" t="s">
+      <c r="L10" s="12" t="s">
         <v>463</v>
       </c>
-      <c r="N10" s="11" t="s">
+      <c r="N10" s="12" t="s">
         <v>464</v>
       </c>
-      <c r="O10" s="11" t="s">
+      <c r="O10" s="12" t="s">
         <v>465</v>
       </c>
-      <c r="P10" s="11" t="s">
+      <c r="P10" s="12" t="s">
         <v>429</v>
       </c>
-      <c r="Y10" s="11" t="s">
+      <c r="Y10" s="12" t="s">
         <v>466</v>
       </c>
-      <c r="AC10" s="11" t="s">
+      <c r="AC10" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AD10" s="11" t="s">
+      <c r="AD10" s="12" t="s">
         <v>467</v>
       </c>
-      <c r="AE10" s="11" t="s">
+      <c r="AE10" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AF10" s="11" t="s">
+      <c r="AF10" s="12" t="s">
         <v>468</v>
       </c>
-      <c r="AG10" s="11" t="s">
+      <c r="AG10" s="12" t="s">
         <v>469</v>
       </c>
-      <c r="AH10" s="11" t="s">
+      <c r="AH10" s="12" t="s">
         <v>438</v>
       </c>
-      <c r="AI10" s="11" t="s">
+      <c r="AI10" s="12" t="s">
         <v>470</v>
       </c>
-      <c r="AJ10" s="11" t="s">
+      <c r="AJ10" s="12" t="s">
         <v>471</v>
       </c>
       <c r="AK10" s="19"/>
-      <c r="AL10" s="11" t="s">
+      <c r="AL10" s="12" t="s">
         <v>457</v>
       </c>
-      <c r="AM10" s="11" t="s">
+      <c r="AM10" s="12" t="s">
         <v>440</v>
       </c>
       <c r="AN10" s="19"/>
-      <c r="AO10" s="11" t="s">
+      <c r="AO10" s="12" t="s">
         <v>472</v>
       </c>
       <c r="AP10" s="19"/>
       <c r="AQ10" s="19"/>
-      <c r="AR10" s="11" t="s">
+      <c r="AR10" s="12" t="s">
         <v>473</v>
       </c>
-      <c r="AS10" s="11" t="s">
+      <c r="AS10" s="12" t="s">
         <v>442</v>
       </c>
-      <c r="AT10" s="11" t="s">
+      <c r="AT10" s="12" t="s">
         <v>443</v>
       </c>
-      <c r="AU10" s="11" t="s">
+      <c r="AU10" s="12" t="s">
         <v>444</v>
       </c>
     </row>
     <row r="11" spans="1:47" ht="40" customHeight="1">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="12" t="s">
         <v>459</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="12" t="s">
         <v>474</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="12" t="s">
         <v>475</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="12" t="s">
         <v>476</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="12" t="s">
         <v>427</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="12" t="s">
         <v>477</v>
       </c>
-      <c r="H11" s="11" t="s">
+      <c r="H11" s="12" t="s">
         <v>429</v>
       </c>
-      <c r="K11" s="11" t="s">
+      <c r="K11" s="12" t="s">
         <v>463</v>
       </c>
-      <c r="L11" s="11" t="s">
+      <c r="L11" s="12" t="s">
         <v>478</v>
       </c>
-      <c r="N11" s="11" t="s">
+      <c r="N11" s="12" t="s">
         <v>479</v>
       </c>
-      <c r="O11" s="11" t="s">
+      <c r="O11" s="12" t="s">
         <v>480</v>
       </c>
-      <c r="P11" s="11" t="s">
+      <c r="P11" s="12" t="s">
         <v>429</v>
       </c>
-      <c r="Y11" s="11" t="s">
+      <c r="Y11" s="12" t="s">
         <v>481</v>
       </c>
-      <c r="AC11" s="11" t="s">
+      <c r="AC11" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AD11" s="11" t="s">
+      <c r="AD11" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AE11" s="11" t="s">
+      <c r="AE11" s="12" t="s">
         <v>467</v>
       </c>
-      <c r="AF11" s="11" t="s">
+      <c r="AF11" s="12" t="s">
         <v>468</v>
       </c>
-      <c r="AG11" s="11" t="s">
+      <c r="AG11" s="12" t="s">
         <v>482</v>
       </c>
-      <c r="AH11" s="11" t="s">
+      <c r="AH11" s="12" t="s">
         <v>438</v>
       </c>
       <c r="AI11" s="19"/>
-      <c r="AJ11" s="11" t="s">
+      <c r="AJ11" s="12" t="s">
         <v>471</v>
       </c>
       <c r="AK11" s="19"/>
@@ -18005,85 +18018,85 @@
       <c r="AM11" s="19"/>
       <c r="AN11" s="19"/>
       <c r="AO11" s="19"/>
-      <c r="AP11" s="11" t="s">
+      <c r="AP11" s="12" t="s">
         <v>483</v>
       </c>
-      <c r="AQ11" s="11" t="s">
+      <c r="AQ11" s="12" t="s">
         <v>483</v>
       </c>
-      <c r="AR11" s="11" t="s">
+      <c r="AR11" s="12" t="s">
         <v>484</v>
       </c>
-      <c r="AS11" s="11" t="s">
+      <c r="AS11" s="12" t="s">
         <v>442</v>
       </c>
-      <c r="AT11" s="11" t="s">
+      <c r="AT11" s="12" t="s">
         <v>443</v>
       </c>
-      <c r="AU11" s="11" t="s">
+      <c r="AU11" s="12" t="s">
         <v>444</v>
       </c>
     </row>
     <row r="12" spans="1:47" ht="40" customHeight="1">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="12" t="s">
         <v>459</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="12" t="s">
         <v>474</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="12" t="s">
         <v>475</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="12" t="s">
         <v>476</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="12" t="s">
         <v>427</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="G12" s="12" t="s">
         <v>485</v>
       </c>
-      <c r="H12" s="11" t="s">
+      <c r="H12" s="12" t="s">
         <v>429</v>
       </c>
-      <c r="K12" s="11" t="s">
+      <c r="K12" s="12" t="s">
         <v>463</v>
       </c>
-      <c r="L12" s="11" t="s">
+      <c r="L12" s="12" t="s">
         <v>478</v>
       </c>
-      <c r="N12" s="11" t="s">
+      <c r="N12" s="12" t="s">
         <v>486</v>
       </c>
-      <c r="O12" s="11" t="s">
+      <c r="O12" s="12" t="s">
         <v>487</v>
       </c>
-      <c r="P12" s="11" t="s">
+      <c r="P12" s="12" t="s">
         <v>488</v>
       </c>
-      <c r="Y12" s="11" t="s">
+      <c r="Y12" s="12" t="s">
         <v>481</v>
       </c>
-      <c r="AC12" s="11" t="s">
+      <c r="AC12" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AD12" s="11" t="s">
+      <c r="AD12" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="AE12" s="11" t="s">
+      <c r="AE12" s="12" t="s">
         <v>467</v>
       </c>
-      <c r="AF12" s="11" t="s">
+      <c r="AF12" s="12" t="s">
         <v>468</v>
       </c>
-      <c r="AG12" s="11" t="s">
+      <c r="AG12" s="12" t="s">
         <v>482</v>
       </c>
-      <c r="AH12" s="11" t="s">
+      <c r="AH12" s="12" t="s">
         <v>438</v>
       </c>
       <c r="AI12" s="19"/>
-      <c r="AJ12" s="11" t="s">
+      <c r="AJ12" s="12" t="s">
         <v>471</v>
       </c>
       <c r="AK12" s="19"/>
@@ -18091,21 +18104,425 @@
       <c r="AM12" s="19"/>
       <c r="AN12" s="19"/>
       <c r="AO12" s="19"/>
-      <c r="AR12" s="11" t="s">
+      <c r="AR12" s="12" t="s">
         <v>489</v>
       </c>
-      <c r="AS12" s="11" t="s">
+      <c r="AS12" s="12" t="s">
         <v>442</v>
       </c>
-      <c r="AT12" s="11" t="s">
+      <c r="AT12" s="12" t="s">
         <v>443</v>
       </c>
-      <c r="AU12" s="11" t="s">
+      <c r="AU12" s="12" t="s">
         <v>444</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="428">
+    <mergeCell ref="AT11"/>
+    <mergeCell ref="AT12"/>
+    <mergeCell ref="AU1"/>
+    <mergeCell ref="AU3"/>
+    <mergeCell ref="AU4"/>
+    <mergeCell ref="AU5"/>
+    <mergeCell ref="AU6"/>
+    <mergeCell ref="AU7"/>
+    <mergeCell ref="AU8"/>
+    <mergeCell ref="AU9"/>
+    <mergeCell ref="AU10"/>
+    <mergeCell ref="AU11"/>
+    <mergeCell ref="AU12"/>
+    <mergeCell ref="AT1"/>
+    <mergeCell ref="AT3"/>
+    <mergeCell ref="AT4"/>
+    <mergeCell ref="AT5"/>
+    <mergeCell ref="AT6"/>
+    <mergeCell ref="AT7"/>
+    <mergeCell ref="AT8"/>
+    <mergeCell ref="AT9"/>
+    <mergeCell ref="AT10"/>
+    <mergeCell ref="AR12"/>
+    <mergeCell ref="AS1"/>
+    <mergeCell ref="AS3"/>
+    <mergeCell ref="AS4"/>
+    <mergeCell ref="AS5"/>
+    <mergeCell ref="AS6"/>
+    <mergeCell ref="AS7"/>
+    <mergeCell ref="AS8"/>
+    <mergeCell ref="AS9"/>
+    <mergeCell ref="AS10"/>
+    <mergeCell ref="AS11"/>
+    <mergeCell ref="AS12"/>
+    <mergeCell ref="AQ11"/>
+    <mergeCell ref="AR1"/>
+    <mergeCell ref="AR3"/>
+    <mergeCell ref="AR4"/>
+    <mergeCell ref="AR5"/>
+    <mergeCell ref="AR6"/>
+    <mergeCell ref="AR7"/>
+    <mergeCell ref="AR8"/>
+    <mergeCell ref="AR9"/>
+    <mergeCell ref="AR10"/>
+    <mergeCell ref="AR11"/>
+    <mergeCell ref="AQ1"/>
+    <mergeCell ref="AQ3"/>
+    <mergeCell ref="AQ4"/>
+    <mergeCell ref="AQ5"/>
+    <mergeCell ref="AQ6"/>
+    <mergeCell ref="AQ7"/>
+    <mergeCell ref="AQ8"/>
+    <mergeCell ref="AQ9"/>
+    <mergeCell ref="AQ10"/>
+    <mergeCell ref="AO11"/>
+    <mergeCell ref="AO12"/>
+    <mergeCell ref="AP1"/>
+    <mergeCell ref="AP3"/>
+    <mergeCell ref="AP4"/>
+    <mergeCell ref="AP5"/>
+    <mergeCell ref="AP6"/>
+    <mergeCell ref="AP7"/>
+    <mergeCell ref="AP8"/>
+    <mergeCell ref="AP9"/>
+    <mergeCell ref="AP10"/>
+    <mergeCell ref="AP11"/>
+    <mergeCell ref="AO1"/>
+    <mergeCell ref="AO3"/>
+    <mergeCell ref="AO4"/>
+    <mergeCell ref="AO5"/>
+    <mergeCell ref="AO6"/>
+    <mergeCell ref="AO7"/>
+    <mergeCell ref="AO8"/>
+    <mergeCell ref="AO9"/>
+    <mergeCell ref="AO10"/>
+    <mergeCell ref="AM11"/>
+    <mergeCell ref="AM12"/>
+    <mergeCell ref="AN1"/>
+    <mergeCell ref="AN3"/>
+    <mergeCell ref="AN4"/>
+    <mergeCell ref="AN5"/>
+    <mergeCell ref="AN6"/>
+    <mergeCell ref="AN7"/>
+    <mergeCell ref="AN8"/>
+    <mergeCell ref="AN9"/>
+    <mergeCell ref="AN10"/>
+    <mergeCell ref="AN11"/>
+    <mergeCell ref="AN12"/>
+    <mergeCell ref="AM1"/>
+    <mergeCell ref="AM3"/>
+    <mergeCell ref="AM4"/>
+    <mergeCell ref="AM5"/>
+    <mergeCell ref="AM6"/>
+    <mergeCell ref="AM7"/>
+    <mergeCell ref="AM8"/>
+    <mergeCell ref="AM9"/>
+    <mergeCell ref="AM10"/>
+    <mergeCell ref="AK11"/>
+    <mergeCell ref="AK12"/>
+    <mergeCell ref="AL1"/>
+    <mergeCell ref="AL3"/>
+    <mergeCell ref="AL4"/>
+    <mergeCell ref="AL5"/>
+    <mergeCell ref="AL6"/>
+    <mergeCell ref="AL7"/>
+    <mergeCell ref="AL8"/>
+    <mergeCell ref="AL9"/>
+    <mergeCell ref="AL10"/>
+    <mergeCell ref="AL11"/>
+    <mergeCell ref="AL12"/>
+    <mergeCell ref="AK1"/>
+    <mergeCell ref="AK3"/>
+    <mergeCell ref="AK4"/>
+    <mergeCell ref="AK5"/>
+    <mergeCell ref="AK6"/>
+    <mergeCell ref="AK7"/>
+    <mergeCell ref="AK8"/>
+    <mergeCell ref="AK9"/>
+    <mergeCell ref="AK10"/>
+    <mergeCell ref="AI11"/>
+    <mergeCell ref="AI12"/>
+    <mergeCell ref="AJ1"/>
+    <mergeCell ref="AJ3"/>
+    <mergeCell ref="AJ4"/>
+    <mergeCell ref="AJ5"/>
+    <mergeCell ref="AJ6"/>
+    <mergeCell ref="AJ7"/>
+    <mergeCell ref="AJ8"/>
+    <mergeCell ref="AJ9"/>
+    <mergeCell ref="AJ10"/>
+    <mergeCell ref="AJ11"/>
+    <mergeCell ref="AJ12"/>
+    <mergeCell ref="AI1"/>
+    <mergeCell ref="AI3"/>
+    <mergeCell ref="AI4"/>
+    <mergeCell ref="AI5"/>
+    <mergeCell ref="AI6"/>
+    <mergeCell ref="AI7"/>
+    <mergeCell ref="AI8"/>
+    <mergeCell ref="AI9"/>
+    <mergeCell ref="AI10"/>
+    <mergeCell ref="AG1"/>
+    <mergeCell ref="AG3"/>
+    <mergeCell ref="AG4"/>
+    <mergeCell ref="AG5"/>
+    <mergeCell ref="AG6"/>
+    <mergeCell ref="AG10"/>
+    <mergeCell ref="AG11"/>
+    <mergeCell ref="AG12"/>
+    <mergeCell ref="AH1"/>
+    <mergeCell ref="AH3"/>
+    <mergeCell ref="AH4"/>
+    <mergeCell ref="AH5"/>
+    <mergeCell ref="AH6"/>
+    <mergeCell ref="AH7"/>
+    <mergeCell ref="AH8"/>
+    <mergeCell ref="AH9"/>
+    <mergeCell ref="AH10"/>
+    <mergeCell ref="AH11"/>
+    <mergeCell ref="AH12"/>
+    <mergeCell ref="AE11"/>
+    <mergeCell ref="AE12"/>
+    <mergeCell ref="AF1"/>
+    <mergeCell ref="AF3"/>
+    <mergeCell ref="AF4"/>
+    <mergeCell ref="AF5"/>
+    <mergeCell ref="AF6"/>
+    <mergeCell ref="AF7"/>
+    <mergeCell ref="AF8"/>
+    <mergeCell ref="AF9"/>
+    <mergeCell ref="AF10"/>
+    <mergeCell ref="AF11"/>
+    <mergeCell ref="AF12"/>
+    <mergeCell ref="AE1"/>
+    <mergeCell ref="AE3"/>
+    <mergeCell ref="AE4"/>
+    <mergeCell ref="AE5"/>
+    <mergeCell ref="AE6"/>
+    <mergeCell ref="AE7"/>
+    <mergeCell ref="AE8"/>
+    <mergeCell ref="AE9"/>
+    <mergeCell ref="AE10"/>
+    <mergeCell ref="AC7"/>
+    <mergeCell ref="AC8"/>
+    <mergeCell ref="AC9"/>
+    <mergeCell ref="AC10"/>
+    <mergeCell ref="AC11"/>
+    <mergeCell ref="AC12"/>
+    <mergeCell ref="AD1"/>
+    <mergeCell ref="AD3"/>
+    <mergeCell ref="AD4"/>
+    <mergeCell ref="AD5"/>
+    <mergeCell ref="AD6"/>
+    <mergeCell ref="AD7"/>
+    <mergeCell ref="AD8"/>
+    <mergeCell ref="AD9"/>
+    <mergeCell ref="AD10"/>
+    <mergeCell ref="AD11"/>
+    <mergeCell ref="AD12"/>
+    <mergeCell ref="AB1"/>
+    <mergeCell ref="AB3"/>
+    <mergeCell ref="AB4"/>
+    <mergeCell ref="AB5"/>
+    <mergeCell ref="AB6"/>
+    <mergeCell ref="AC1"/>
+    <mergeCell ref="AC3"/>
+    <mergeCell ref="AC4"/>
+    <mergeCell ref="AC5"/>
+    <mergeCell ref="AC6"/>
+    <mergeCell ref="Y11"/>
+    <mergeCell ref="Y12"/>
+    <mergeCell ref="Z1"/>
+    <mergeCell ref="Z3"/>
+    <mergeCell ref="Z4"/>
+    <mergeCell ref="Z5"/>
+    <mergeCell ref="Z6"/>
+    <mergeCell ref="AA1"/>
+    <mergeCell ref="AA3"/>
+    <mergeCell ref="AA4"/>
+    <mergeCell ref="AA5"/>
+    <mergeCell ref="AA6"/>
+    <mergeCell ref="Y1"/>
+    <mergeCell ref="Y3"/>
+    <mergeCell ref="Y4"/>
+    <mergeCell ref="Y5"/>
+    <mergeCell ref="Y6"/>
+    <mergeCell ref="Y7"/>
+    <mergeCell ref="Y8"/>
+    <mergeCell ref="Y9"/>
+    <mergeCell ref="Y10"/>
+    <mergeCell ref="W1"/>
+    <mergeCell ref="W3"/>
+    <mergeCell ref="W4"/>
+    <mergeCell ref="W5"/>
+    <mergeCell ref="W6"/>
+    <mergeCell ref="X1"/>
+    <mergeCell ref="X3"/>
+    <mergeCell ref="X4"/>
+    <mergeCell ref="X5"/>
+    <mergeCell ref="X6"/>
+    <mergeCell ref="U1"/>
+    <mergeCell ref="U3"/>
+    <mergeCell ref="U4"/>
+    <mergeCell ref="U5"/>
+    <mergeCell ref="U6"/>
+    <mergeCell ref="V1"/>
+    <mergeCell ref="V3"/>
+    <mergeCell ref="V4"/>
+    <mergeCell ref="V5"/>
+    <mergeCell ref="V6"/>
+    <mergeCell ref="S1"/>
+    <mergeCell ref="S3"/>
+    <mergeCell ref="S4"/>
+    <mergeCell ref="S5"/>
+    <mergeCell ref="S6"/>
+    <mergeCell ref="T1"/>
+    <mergeCell ref="T3"/>
+    <mergeCell ref="T4"/>
+    <mergeCell ref="T5"/>
+    <mergeCell ref="T6"/>
+    <mergeCell ref="P11"/>
+    <mergeCell ref="P12"/>
+    <mergeCell ref="Q1"/>
+    <mergeCell ref="Q3"/>
+    <mergeCell ref="Q4"/>
+    <mergeCell ref="Q5"/>
+    <mergeCell ref="Q6"/>
+    <mergeCell ref="R1"/>
+    <mergeCell ref="R3"/>
+    <mergeCell ref="R4"/>
+    <mergeCell ref="R5"/>
+    <mergeCell ref="R6"/>
+    <mergeCell ref="P1"/>
+    <mergeCell ref="P3"/>
+    <mergeCell ref="P4"/>
+    <mergeCell ref="P5"/>
+    <mergeCell ref="P6"/>
+    <mergeCell ref="P7"/>
+    <mergeCell ref="P8"/>
+    <mergeCell ref="P9"/>
+    <mergeCell ref="P10"/>
+    <mergeCell ref="N10"/>
+    <mergeCell ref="N11"/>
+    <mergeCell ref="N12"/>
+    <mergeCell ref="O1"/>
+    <mergeCell ref="O3"/>
+    <mergeCell ref="O4"/>
+    <mergeCell ref="O5"/>
+    <mergeCell ref="O6"/>
+    <mergeCell ref="O7"/>
+    <mergeCell ref="O8"/>
+    <mergeCell ref="O9"/>
+    <mergeCell ref="O10"/>
+    <mergeCell ref="O11"/>
+    <mergeCell ref="O12"/>
+    <mergeCell ref="M1"/>
+    <mergeCell ref="M3"/>
+    <mergeCell ref="M4"/>
+    <mergeCell ref="M5"/>
+    <mergeCell ref="M6"/>
+    <mergeCell ref="M7"/>
+    <mergeCell ref="M8"/>
+    <mergeCell ref="M9"/>
+    <mergeCell ref="N1"/>
+    <mergeCell ref="N3"/>
+    <mergeCell ref="N4"/>
+    <mergeCell ref="N5"/>
+    <mergeCell ref="N6"/>
+    <mergeCell ref="N7"/>
+    <mergeCell ref="N8"/>
+    <mergeCell ref="N9"/>
+    <mergeCell ref="K10"/>
+    <mergeCell ref="K11"/>
+    <mergeCell ref="K12"/>
+    <mergeCell ref="L1"/>
+    <mergeCell ref="L3"/>
+    <mergeCell ref="L4"/>
+    <mergeCell ref="L5"/>
+    <mergeCell ref="L6"/>
+    <mergeCell ref="L7"/>
+    <mergeCell ref="L8"/>
+    <mergeCell ref="L9"/>
+    <mergeCell ref="L10"/>
+    <mergeCell ref="L11"/>
+    <mergeCell ref="L12"/>
+    <mergeCell ref="J1"/>
+    <mergeCell ref="J3"/>
+    <mergeCell ref="J4"/>
+    <mergeCell ref="J5"/>
+    <mergeCell ref="J6"/>
+    <mergeCell ref="J7"/>
+    <mergeCell ref="J8"/>
+    <mergeCell ref="J9"/>
+    <mergeCell ref="K1"/>
+    <mergeCell ref="K3"/>
+    <mergeCell ref="K4"/>
+    <mergeCell ref="K5"/>
+    <mergeCell ref="K6"/>
+    <mergeCell ref="K7"/>
+    <mergeCell ref="K8"/>
+    <mergeCell ref="K9"/>
+    <mergeCell ref="H12"/>
+    <mergeCell ref="I1"/>
+    <mergeCell ref="I3"/>
+    <mergeCell ref="I4"/>
+    <mergeCell ref="I5"/>
+    <mergeCell ref="I6"/>
+    <mergeCell ref="I7"/>
+    <mergeCell ref="I8"/>
+    <mergeCell ref="I9"/>
+    <mergeCell ref="H1"/>
+    <mergeCell ref="H3"/>
+    <mergeCell ref="H4"/>
+    <mergeCell ref="H5"/>
+    <mergeCell ref="H6"/>
+    <mergeCell ref="H7"/>
+    <mergeCell ref="H8"/>
+    <mergeCell ref="H9"/>
+    <mergeCell ref="H11"/>
+    <mergeCell ref="C8"/>
+    <mergeCell ref="F12"/>
+    <mergeCell ref="G1"/>
+    <mergeCell ref="G3"/>
+    <mergeCell ref="G4"/>
+    <mergeCell ref="G5"/>
+    <mergeCell ref="G6"/>
+    <mergeCell ref="G7"/>
+    <mergeCell ref="G8"/>
+    <mergeCell ref="G9"/>
+    <mergeCell ref="G11"/>
+    <mergeCell ref="G12"/>
+    <mergeCell ref="F1"/>
+    <mergeCell ref="F3"/>
+    <mergeCell ref="F4"/>
+    <mergeCell ref="F5"/>
+    <mergeCell ref="F6"/>
+    <mergeCell ref="F7"/>
+    <mergeCell ref="F8"/>
+    <mergeCell ref="F9"/>
+    <mergeCell ref="F11"/>
+    <mergeCell ref="A8"/>
+    <mergeCell ref="C11"/>
+    <mergeCell ref="C12"/>
+    <mergeCell ref="D1"/>
+    <mergeCell ref="D3"/>
+    <mergeCell ref="D4"/>
+    <mergeCell ref="D5"/>
+    <mergeCell ref="D6"/>
+    <mergeCell ref="E1"/>
+    <mergeCell ref="E3"/>
+    <mergeCell ref="E4"/>
+    <mergeCell ref="E5"/>
+    <mergeCell ref="E6"/>
+    <mergeCell ref="E7"/>
+    <mergeCell ref="E8"/>
+    <mergeCell ref="E9"/>
+    <mergeCell ref="E11"/>
+    <mergeCell ref="E12"/>
+    <mergeCell ref="C1"/>
+    <mergeCell ref="C3"/>
+    <mergeCell ref="C4"/>
+    <mergeCell ref="C5"/>
+    <mergeCell ref="C6"/>
+    <mergeCell ref="C7"/>
     <mergeCell ref="A9"/>
     <mergeCell ref="C9"/>
     <mergeCell ref="C10"/>
@@ -18130,410 +18547,6 @@
     <mergeCell ref="A5"/>
     <mergeCell ref="A6"/>
     <mergeCell ref="A7"/>
-    <mergeCell ref="A8"/>
-    <mergeCell ref="C11"/>
-    <mergeCell ref="C12"/>
-    <mergeCell ref="D1"/>
-    <mergeCell ref="D3"/>
-    <mergeCell ref="D4"/>
-    <mergeCell ref="D5"/>
-    <mergeCell ref="D6"/>
-    <mergeCell ref="E1"/>
-    <mergeCell ref="E3"/>
-    <mergeCell ref="E4"/>
-    <mergeCell ref="E5"/>
-    <mergeCell ref="E6"/>
-    <mergeCell ref="E7"/>
-    <mergeCell ref="E8"/>
-    <mergeCell ref="E9"/>
-    <mergeCell ref="E11"/>
-    <mergeCell ref="E12"/>
-    <mergeCell ref="C1"/>
-    <mergeCell ref="C3"/>
-    <mergeCell ref="C4"/>
-    <mergeCell ref="C5"/>
-    <mergeCell ref="C6"/>
-    <mergeCell ref="C7"/>
-    <mergeCell ref="C8"/>
-    <mergeCell ref="F12"/>
-    <mergeCell ref="G1"/>
-    <mergeCell ref="G3"/>
-    <mergeCell ref="G4"/>
-    <mergeCell ref="G5"/>
-    <mergeCell ref="G6"/>
-    <mergeCell ref="G7"/>
-    <mergeCell ref="G8"/>
-    <mergeCell ref="G9"/>
-    <mergeCell ref="G11"/>
-    <mergeCell ref="G12"/>
-    <mergeCell ref="F1"/>
-    <mergeCell ref="F3"/>
-    <mergeCell ref="F4"/>
-    <mergeCell ref="F5"/>
-    <mergeCell ref="F6"/>
-    <mergeCell ref="F7"/>
-    <mergeCell ref="F8"/>
-    <mergeCell ref="F9"/>
-    <mergeCell ref="F11"/>
-    <mergeCell ref="H12"/>
-    <mergeCell ref="I1"/>
-    <mergeCell ref="I3"/>
-    <mergeCell ref="I4"/>
-    <mergeCell ref="I5"/>
-    <mergeCell ref="I6"/>
-    <mergeCell ref="I7"/>
-    <mergeCell ref="I8"/>
-    <mergeCell ref="I9"/>
-    <mergeCell ref="H1"/>
-    <mergeCell ref="H3"/>
-    <mergeCell ref="H4"/>
-    <mergeCell ref="H5"/>
-    <mergeCell ref="H6"/>
-    <mergeCell ref="H7"/>
-    <mergeCell ref="H8"/>
-    <mergeCell ref="H9"/>
-    <mergeCell ref="H11"/>
-    <mergeCell ref="J1"/>
-    <mergeCell ref="J3"/>
-    <mergeCell ref="J4"/>
-    <mergeCell ref="J5"/>
-    <mergeCell ref="J6"/>
-    <mergeCell ref="J7"/>
-    <mergeCell ref="J8"/>
-    <mergeCell ref="J9"/>
-    <mergeCell ref="K1"/>
-    <mergeCell ref="K3"/>
-    <mergeCell ref="K4"/>
-    <mergeCell ref="K5"/>
-    <mergeCell ref="K6"/>
-    <mergeCell ref="K7"/>
-    <mergeCell ref="K8"/>
-    <mergeCell ref="K9"/>
-    <mergeCell ref="K10"/>
-    <mergeCell ref="K11"/>
-    <mergeCell ref="K12"/>
-    <mergeCell ref="L1"/>
-    <mergeCell ref="L3"/>
-    <mergeCell ref="L4"/>
-    <mergeCell ref="L5"/>
-    <mergeCell ref="L6"/>
-    <mergeCell ref="L7"/>
-    <mergeCell ref="L8"/>
-    <mergeCell ref="L9"/>
-    <mergeCell ref="L10"/>
-    <mergeCell ref="L11"/>
-    <mergeCell ref="L12"/>
-    <mergeCell ref="M1"/>
-    <mergeCell ref="M3"/>
-    <mergeCell ref="M4"/>
-    <mergeCell ref="M5"/>
-    <mergeCell ref="M6"/>
-    <mergeCell ref="M7"/>
-    <mergeCell ref="M8"/>
-    <mergeCell ref="M9"/>
-    <mergeCell ref="N1"/>
-    <mergeCell ref="N3"/>
-    <mergeCell ref="N4"/>
-    <mergeCell ref="N5"/>
-    <mergeCell ref="N6"/>
-    <mergeCell ref="N7"/>
-    <mergeCell ref="N8"/>
-    <mergeCell ref="N9"/>
-    <mergeCell ref="N10"/>
-    <mergeCell ref="N11"/>
-    <mergeCell ref="N12"/>
-    <mergeCell ref="O1"/>
-    <mergeCell ref="O3"/>
-    <mergeCell ref="O4"/>
-    <mergeCell ref="O5"/>
-    <mergeCell ref="O6"/>
-    <mergeCell ref="O7"/>
-    <mergeCell ref="O8"/>
-    <mergeCell ref="O9"/>
-    <mergeCell ref="O10"/>
-    <mergeCell ref="O11"/>
-    <mergeCell ref="O12"/>
-    <mergeCell ref="P11"/>
-    <mergeCell ref="P12"/>
-    <mergeCell ref="Q1"/>
-    <mergeCell ref="Q3"/>
-    <mergeCell ref="Q4"/>
-    <mergeCell ref="Q5"/>
-    <mergeCell ref="Q6"/>
-    <mergeCell ref="R1"/>
-    <mergeCell ref="R3"/>
-    <mergeCell ref="R4"/>
-    <mergeCell ref="R5"/>
-    <mergeCell ref="R6"/>
-    <mergeCell ref="P1"/>
-    <mergeCell ref="P3"/>
-    <mergeCell ref="P4"/>
-    <mergeCell ref="P5"/>
-    <mergeCell ref="P6"/>
-    <mergeCell ref="P7"/>
-    <mergeCell ref="P8"/>
-    <mergeCell ref="P9"/>
-    <mergeCell ref="P10"/>
-    <mergeCell ref="S1"/>
-    <mergeCell ref="S3"/>
-    <mergeCell ref="S4"/>
-    <mergeCell ref="S5"/>
-    <mergeCell ref="S6"/>
-    <mergeCell ref="T1"/>
-    <mergeCell ref="T3"/>
-    <mergeCell ref="T4"/>
-    <mergeCell ref="T5"/>
-    <mergeCell ref="T6"/>
-    <mergeCell ref="U1"/>
-    <mergeCell ref="U3"/>
-    <mergeCell ref="U4"/>
-    <mergeCell ref="U5"/>
-    <mergeCell ref="U6"/>
-    <mergeCell ref="V1"/>
-    <mergeCell ref="V3"/>
-    <mergeCell ref="V4"/>
-    <mergeCell ref="V5"/>
-    <mergeCell ref="V6"/>
-    <mergeCell ref="W1"/>
-    <mergeCell ref="W3"/>
-    <mergeCell ref="W4"/>
-    <mergeCell ref="W5"/>
-    <mergeCell ref="W6"/>
-    <mergeCell ref="X1"/>
-    <mergeCell ref="X3"/>
-    <mergeCell ref="X4"/>
-    <mergeCell ref="X5"/>
-    <mergeCell ref="X6"/>
-    <mergeCell ref="Y11"/>
-    <mergeCell ref="Y12"/>
-    <mergeCell ref="Z1"/>
-    <mergeCell ref="Z3"/>
-    <mergeCell ref="Z4"/>
-    <mergeCell ref="Z5"/>
-    <mergeCell ref="Z6"/>
-    <mergeCell ref="AA1"/>
-    <mergeCell ref="AA3"/>
-    <mergeCell ref="AA4"/>
-    <mergeCell ref="AA5"/>
-    <mergeCell ref="AA6"/>
-    <mergeCell ref="Y1"/>
-    <mergeCell ref="Y3"/>
-    <mergeCell ref="Y4"/>
-    <mergeCell ref="Y5"/>
-    <mergeCell ref="Y6"/>
-    <mergeCell ref="Y7"/>
-    <mergeCell ref="Y8"/>
-    <mergeCell ref="Y9"/>
-    <mergeCell ref="Y10"/>
-    <mergeCell ref="AB1"/>
-    <mergeCell ref="AB3"/>
-    <mergeCell ref="AB4"/>
-    <mergeCell ref="AB5"/>
-    <mergeCell ref="AB6"/>
-    <mergeCell ref="AC1"/>
-    <mergeCell ref="AC3"/>
-    <mergeCell ref="AC4"/>
-    <mergeCell ref="AC5"/>
-    <mergeCell ref="AC6"/>
-    <mergeCell ref="AC7"/>
-    <mergeCell ref="AC8"/>
-    <mergeCell ref="AC9"/>
-    <mergeCell ref="AC10"/>
-    <mergeCell ref="AC11"/>
-    <mergeCell ref="AC12"/>
-    <mergeCell ref="AD1"/>
-    <mergeCell ref="AD3"/>
-    <mergeCell ref="AD4"/>
-    <mergeCell ref="AD5"/>
-    <mergeCell ref="AD6"/>
-    <mergeCell ref="AD7"/>
-    <mergeCell ref="AD8"/>
-    <mergeCell ref="AD9"/>
-    <mergeCell ref="AD10"/>
-    <mergeCell ref="AD11"/>
-    <mergeCell ref="AD12"/>
-    <mergeCell ref="AE11"/>
-    <mergeCell ref="AE12"/>
-    <mergeCell ref="AF1"/>
-    <mergeCell ref="AF3"/>
-    <mergeCell ref="AF4"/>
-    <mergeCell ref="AF5"/>
-    <mergeCell ref="AF6"/>
-    <mergeCell ref="AF7"/>
-    <mergeCell ref="AF8"/>
-    <mergeCell ref="AF9"/>
-    <mergeCell ref="AF10"/>
-    <mergeCell ref="AF11"/>
-    <mergeCell ref="AF12"/>
-    <mergeCell ref="AE1"/>
-    <mergeCell ref="AE3"/>
-    <mergeCell ref="AE4"/>
-    <mergeCell ref="AE5"/>
-    <mergeCell ref="AE6"/>
-    <mergeCell ref="AE7"/>
-    <mergeCell ref="AE8"/>
-    <mergeCell ref="AE9"/>
-    <mergeCell ref="AE10"/>
-    <mergeCell ref="AG1"/>
-    <mergeCell ref="AG3"/>
-    <mergeCell ref="AG4"/>
-    <mergeCell ref="AG5"/>
-    <mergeCell ref="AG6"/>
-    <mergeCell ref="AG10"/>
-    <mergeCell ref="AG11"/>
-    <mergeCell ref="AG12"/>
-    <mergeCell ref="AH1"/>
-    <mergeCell ref="AH3"/>
-    <mergeCell ref="AH4"/>
-    <mergeCell ref="AH5"/>
-    <mergeCell ref="AH6"/>
-    <mergeCell ref="AH7"/>
-    <mergeCell ref="AH8"/>
-    <mergeCell ref="AH9"/>
-    <mergeCell ref="AH10"/>
-    <mergeCell ref="AH11"/>
-    <mergeCell ref="AH12"/>
-    <mergeCell ref="AI11"/>
-    <mergeCell ref="AI12"/>
-    <mergeCell ref="AJ1"/>
-    <mergeCell ref="AJ3"/>
-    <mergeCell ref="AJ4"/>
-    <mergeCell ref="AJ5"/>
-    <mergeCell ref="AJ6"/>
-    <mergeCell ref="AJ7"/>
-    <mergeCell ref="AJ8"/>
-    <mergeCell ref="AJ9"/>
-    <mergeCell ref="AJ10"/>
-    <mergeCell ref="AJ11"/>
-    <mergeCell ref="AJ12"/>
-    <mergeCell ref="AI1"/>
-    <mergeCell ref="AI3"/>
-    <mergeCell ref="AI4"/>
-    <mergeCell ref="AI5"/>
-    <mergeCell ref="AI6"/>
-    <mergeCell ref="AI7"/>
-    <mergeCell ref="AI8"/>
-    <mergeCell ref="AI9"/>
-    <mergeCell ref="AI10"/>
-    <mergeCell ref="AK11"/>
-    <mergeCell ref="AK12"/>
-    <mergeCell ref="AL1"/>
-    <mergeCell ref="AL3"/>
-    <mergeCell ref="AL4"/>
-    <mergeCell ref="AL5"/>
-    <mergeCell ref="AL6"/>
-    <mergeCell ref="AL7"/>
-    <mergeCell ref="AL8"/>
-    <mergeCell ref="AL9"/>
-    <mergeCell ref="AL10"/>
-    <mergeCell ref="AL11"/>
-    <mergeCell ref="AL12"/>
-    <mergeCell ref="AK1"/>
-    <mergeCell ref="AK3"/>
-    <mergeCell ref="AK4"/>
-    <mergeCell ref="AK5"/>
-    <mergeCell ref="AK6"/>
-    <mergeCell ref="AK7"/>
-    <mergeCell ref="AK8"/>
-    <mergeCell ref="AK9"/>
-    <mergeCell ref="AK10"/>
-    <mergeCell ref="AM11"/>
-    <mergeCell ref="AM12"/>
-    <mergeCell ref="AN1"/>
-    <mergeCell ref="AN3"/>
-    <mergeCell ref="AN4"/>
-    <mergeCell ref="AN5"/>
-    <mergeCell ref="AN6"/>
-    <mergeCell ref="AN7"/>
-    <mergeCell ref="AN8"/>
-    <mergeCell ref="AN9"/>
-    <mergeCell ref="AN10"/>
-    <mergeCell ref="AN11"/>
-    <mergeCell ref="AN12"/>
-    <mergeCell ref="AM1"/>
-    <mergeCell ref="AM3"/>
-    <mergeCell ref="AM4"/>
-    <mergeCell ref="AM5"/>
-    <mergeCell ref="AM6"/>
-    <mergeCell ref="AM7"/>
-    <mergeCell ref="AM8"/>
-    <mergeCell ref="AM9"/>
-    <mergeCell ref="AM10"/>
-    <mergeCell ref="AO11"/>
-    <mergeCell ref="AO12"/>
-    <mergeCell ref="AP1"/>
-    <mergeCell ref="AP3"/>
-    <mergeCell ref="AP4"/>
-    <mergeCell ref="AP5"/>
-    <mergeCell ref="AP6"/>
-    <mergeCell ref="AP7"/>
-    <mergeCell ref="AP8"/>
-    <mergeCell ref="AP9"/>
-    <mergeCell ref="AP10"/>
-    <mergeCell ref="AP11"/>
-    <mergeCell ref="AO1"/>
-    <mergeCell ref="AO3"/>
-    <mergeCell ref="AO4"/>
-    <mergeCell ref="AO5"/>
-    <mergeCell ref="AO6"/>
-    <mergeCell ref="AO7"/>
-    <mergeCell ref="AO8"/>
-    <mergeCell ref="AO9"/>
-    <mergeCell ref="AO10"/>
-    <mergeCell ref="AQ11"/>
-    <mergeCell ref="AR1"/>
-    <mergeCell ref="AR3"/>
-    <mergeCell ref="AR4"/>
-    <mergeCell ref="AR5"/>
-    <mergeCell ref="AR6"/>
-    <mergeCell ref="AR7"/>
-    <mergeCell ref="AR8"/>
-    <mergeCell ref="AR9"/>
-    <mergeCell ref="AR10"/>
-    <mergeCell ref="AR11"/>
-    <mergeCell ref="AQ1"/>
-    <mergeCell ref="AQ3"/>
-    <mergeCell ref="AQ4"/>
-    <mergeCell ref="AQ5"/>
-    <mergeCell ref="AQ6"/>
-    <mergeCell ref="AQ7"/>
-    <mergeCell ref="AQ8"/>
-    <mergeCell ref="AQ9"/>
-    <mergeCell ref="AQ10"/>
-    <mergeCell ref="AR12"/>
-    <mergeCell ref="AS1"/>
-    <mergeCell ref="AS3"/>
-    <mergeCell ref="AS4"/>
-    <mergeCell ref="AS5"/>
-    <mergeCell ref="AS6"/>
-    <mergeCell ref="AS7"/>
-    <mergeCell ref="AS8"/>
-    <mergeCell ref="AS9"/>
-    <mergeCell ref="AS10"/>
-    <mergeCell ref="AS11"/>
-    <mergeCell ref="AS12"/>
-    <mergeCell ref="AT11"/>
-    <mergeCell ref="AT12"/>
-    <mergeCell ref="AU1"/>
-    <mergeCell ref="AU3"/>
-    <mergeCell ref="AU4"/>
-    <mergeCell ref="AU5"/>
-    <mergeCell ref="AU6"/>
-    <mergeCell ref="AU7"/>
-    <mergeCell ref="AU8"/>
-    <mergeCell ref="AU9"/>
-    <mergeCell ref="AU10"/>
-    <mergeCell ref="AU11"/>
-    <mergeCell ref="AU12"/>
-    <mergeCell ref="AT1"/>
-    <mergeCell ref="AT3"/>
-    <mergeCell ref="AT4"/>
-    <mergeCell ref="AT5"/>
-    <mergeCell ref="AT6"/>
-    <mergeCell ref="AT7"/>
-    <mergeCell ref="AT8"/>
-    <mergeCell ref="AT9"/>
-    <mergeCell ref="AT10"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>